<commit_message>
chore: regenerate the filled workbook with the clean-vial cherry-pick and raw-cell binaries
Produced by label_terpenos.py + fill_ternarios.py at 81dd2e2. Exports at this
commit: ternarios_resultados.csv changes D2 Superior, F5 Inferior, I2 Superior
(dropped_replicate); binarios_tielines.csv changes the aqueous endpoints of
B, C, F, H and the H organic endpoint (water 0.047 -> 0.017).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TH6VsmAPvEQ8gbxik9hbAj
</commit_message>
<xml_diff>
--- a/Sistemas ternarios_MF_filled.xlsx
+++ b/Sistemas ternarios_MF_filled.xlsx
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AA21" s="2" t="n">
         <f aca="false">SUM(W21:Z21)</f>
-        <v>0.88041091021879</v>
+        <v>0.880410910218789</v>
       </c>
       <c r="AD21" s="0" t="n">
         <v>0.685652539748668</v>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="AA25" s="1" t="n">
         <f aca="false">SUM(W25:Z25)</f>
-        <v>0.985790682882599</v>
+        <v>0.9857906828826</v>
       </c>
       <c r="AE25" s="1" t="n">
         <f aca="false">IFERROR(X25/$AA25,"")</f>
@@ -8636,16 +8636,16 @@
         <v>0.985430521099807</v>
       </c>
       <c r="AD9" s="0" t="n">
-        <v>0.000590019836661907</v>
+        <v>0.000560526618987546</v>
       </c>
       <c r="AE9" s="0" t="n">
-        <v>0.00206682518392184</v>
+        <v>0.000893478724842093</v>
       </c>
       <c r="AF9" s="0" t="n">
-        <v>0.00245617607922325</v>
+        <v>0.00118885241040632</v>
       </c>
       <c r="AG9" s="0" t="n">
-        <v>0.994886978900193</v>
+        <v>0.997357142245764</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14536,16 +14536,16 @@
         <v>0.996292125260283</v>
       </c>
       <c r="AD23" s="0" t="n">
-        <v>0.00587146129699683</v>
+        <v>0.00521925283446224</v>
       </c>
       <c r="AE23" s="0" t="n">
-        <v>0.00238389021032173</v>
+        <v>0.00205635989547664</v>
       </c>
       <c r="AF23" s="0" t="n">
-        <v>0.00218277375296413</v>
+        <v>0.00187613108534968</v>
       </c>
       <c r="AG23" s="0" t="n">
-        <v>0.989561874739717</v>
+        <v>0.990848256184711</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17853,16 +17853,16 @@
         <v>0.994753153749433</v>
       </c>
       <c r="AD9" s="0" t="n">
-        <v>0.000837183649694847</v>
+        <v>0.000623361408690674</v>
       </c>
       <c r="AE9" s="0" t="n">
-        <v>0.0025074574284368</v>
+        <v>0.000780780912192686</v>
       </c>
       <c r="AF9" s="0" t="n">
-        <v>0.0026575126713012</v>
+        <v>0.00073745644692363</v>
       </c>
       <c r="AG9" s="0" t="n">
-        <v>0.993997846250567</v>
+        <v>0.997858401232193</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>